<commit_message>
Implement Milestone 3 career companion features
</commit_message>
<xml_diff>
--- a/docs/project_tracking/Defect_Tracker Template_v0.1.xlsx
+++ b/docs/project_tracking/Defect_Tracker Template_v0.1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bibi Fatima\Downloads\Internship_artifacts\Internship_artifacts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\infosys\ai-career-companion\docs\project_tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DCE2A2-4CA0-420E-A364-3F9C37102532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE39FC11-C11C-4DF5-A54B-ECDED7BB2D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
   <si>
     <t>Sl No</t>
   </si>
@@ -153,6 +153,54 @@
   </si>
   <si>
     <t>Redesigned dashboard integrated with project backend</t>
+  </si>
+  <si>
+    <t>Skill Gap endpoint initially rejected requests when an invalid or placeholder job ID was provided</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>API / Validation</t>
+  </si>
+  <si>
+    <t>Tested the endpoint with valid job IDs returned by the job-matching service and integrated job selection with the skill-gap workflow</t>
+  </si>
+  <si>
+    <t>Skill gap analysis now uses the selected job from current job matches</t>
+  </si>
+  <si>
+    <t>Skill Gap page was not integrated with the selected recommended job</t>
+  </si>
+  <si>
+    <t>Connected recommended job selection to the Skill Gap API and added job-specific analysis flow</t>
+  </si>
+  <si>
+    <t>Selected job ID is passed to the skill-gap endpoint</t>
+  </si>
+  <si>
+    <t>Existing frontend UI was visually basic and did not clearly expose M3 career features</t>
+  </si>
+  <si>
+    <t>UI / UX</t>
+  </si>
+  <si>
+    <t>Redesigned the Career Companion interface with dashboard cards, improved navigation, job details and M3 feature sections</t>
+  </si>
+  <si>
+    <t>Updated UI provides a more professional AI career platform experience</t>
+  </si>
+  <si>
+    <t>M3 feature sections such as Skill Gap, Application Studio and Interview Preparation were displayed only as placeholders</t>
+  </si>
+  <si>
+    <t>Feature Integration</t>
+  </si>
+  <si>
+    <t>Added M3 feature navigation and prepared the interface for Skill Gap, Application Studio and Interview Preparation workflows</t>
+  </si>
+  <si>
+    <t>M3 modules are exposed through the redesigned Career Companion interface</t>
   </si>
 </sst>
 </file>
@@ -258,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -279,6 +327,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -845,57 +899,145 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="6"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="6"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+    <row r="8" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="10">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="11">
+        <v>46287</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="11">
+        <v>46287</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A9" s="10">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="11">
+        <v>46287</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46287</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="11">
+        <v>46288</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" s="11">
+        <v>46288</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="10">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="11">
+        <v>46288</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I11" s="11">
+        <v>46288</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
@@ -1026,7 +1168,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1 G8:G1048576</xm:sqref>
+          <xm:sqref>G1 G12:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1071,21 +1213,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1217,24 +1344,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1250,4 +1375,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
docs: update M4 test cases
</commit_message>
<xml_diff>
--- a/docs/project_tracking/Defect_Tracker Template_v0.1.xlsx
+++ b/docs/project_tracking/Defect_Tracker Template_v0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\infosys\ai-career-companion\docs\project_tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE39FC11-C11C-4DF5-A54B-ECDED7BB2D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F28DA5C-3B9E-4F78-93A0-4CDD0CFB760A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="105">
   <si>
     <t>Sl No</t>
   </si>
@@ -201,13 +201,148 @@
   </si>
   <si>
     <t>M3 modules are exposed through the redesigned Career Companion interface</t>
+  </si>
+  <si>
+    <t>Application Tracker initially required validation for application records before saving them to the database</t>
+  </si>
+  <si>
+    <t>M4</t>
+  </si>
+  <si>
+    <t>Added validation for required application fields and tested application creation with valid and invalid inputs</t>
+  </si>
+  <si>
+    <t>Application records are now validated before persistence</t>
+  </si>
+  <si>
+    <t>Application status changes were not initially reflected consistently across the tracker dashboard</t>
+  </si>
+  <si>
+    <t>Application Workflow</t>
+  </si>
+  <si>
+    <t>Updated application status handling and synchronized status changes with dashboard statistics</t>
+  </si>
+  <si>
+    <t>Application lifecycle status and dashboard counts remain synchronized</t>
+  </si>
+  <si>
+    <t>Application tracker required support for multiple lifecycle stages such as Saved, Applied, Under Review, Shortlisted and Interview Scheduled</t>
+  </si>
+  <si>
+    <t>Implemented and tested the complete application status workflow including Offer Received, Rejected and Withdrawn states</t>
+  </si>
+  <si>
+    <t>Complete application lifecycle is available in the tracker</t>
+  </si>
+  <si>
+    <t>Deadline filtering required separate handling for upcoming, overdue and applications without deadlines</t>
+  </si>
+  <si>
+    <t>Filtering / Validation</t>
+  </si>
+  <si>
+    <t>Added deadline-based filtering and date validation for application records</t>
+  </si>
+  <si>
+    <t>Users can filter applications by deadline status</t>
+  </si>
+  <si>
+    <t>Application dashboard statistics did not initially cover all required application states</t>
+  </si>
+  <si>
+    <t>Dashboard / Data Consistency</t>
+  </si>
+  <si>
+    <t>Updated dashboard aggregation logic to calculate total, active, deadline, interview, offer and rejection counts</t>
+  </si>
+  <si>
+    <t>Dashboard provides consolidated application pipeline metrics</t>
+  </si>
+  <si>
+    <t>Tailored Resume generation required job-specific candidate information to avoid generic application content</t>
+  </si>
+  <si>
+    <t>AI / Feature Integration</t>
+  </si>
+  <si>
+    <t>Connected selected job requirements and verified candidate profile information to the tailored resume workflow</t>
+  </si>
+  <si>
+    <t>Tailored resume generation uses selected job context and candidate profile data</t>
+  </si>
+  <si>
+    <t>Generated application content required protection against unsupported skills, achievements and experience</t>
+  </si>
+  <si>
+    <t>AI / Data Integrity</t>
+  </si>
+  <si>
+    <t>Applied candidate-profile-based prompting and validation rules to restrict generated content to verified information</t>
+  </si>
+  <si>
+    <t>Application materials are designed to avoid unsupported candidate claims</t>
+  </si>
+  <si>
+    <t>Personalized Cover Letter workflow required integration with the selected application and target job</t>
+  </si>
+  <si>
+    <t>Integrated selected job, candidate profile and application context into the cover letter generation workflow</t>
+  </si>
+  <si>
+    <t>Cover letters are generated using job-specific application context</t>
+  </si>
+  <si>
+    <t>Application Tracker actions such as View, Edit and Delete required backend synchronization</t>
+  </si>
+  <si>
+    <t>Connected tracker actions with the corresponding backend application APIs and tested CRUD operations</t>
+  </si>
+  <si>
+    <t>Application records can be viewed, updated and removed through the interface</t>
+  </si>
+  <si>
+    <t>Interview schedule information required integration with tracked application records</t>
+  </si>
+  <si>
+    <t>Application / Interview Integration</t>
+  </si>
+  <si>
+    <t>Added interview scheduling information to application records and integrated it with application tracking</t>
+  </si>
+  <si>
+    <t>Interview information can be associated with the corresponding application</t>
+  </si>
+  <si>
+    <t>Application Tracker required verification of complete end-to-end application management workflow</t>
+  </si>
+  <si>
+    <t>End-to-End Testing</t>
+  </si>
+  <si>
+    <t>Tested application creation, status updates, filtering, deadline handling, editing, deletion and dashboard statistics</t>
+  </si>
+  <si>
+    <t>Application management workflow validated successfully</t>
+  </si>
+  <si>
+    <t>M4 Application Tracker and Studio required final integration testing with existing M1-M3 modules</t>
+  </si>
+  <si>
+    <t>System Integration</t>
+  </si>
+  <si>
+    <t>Performed end-to-end integration testing across profile, resume, job matching, skill gap, application studio and interview workflows</t>
+  </si>
+  <si>
+    <t>M4 functionality integrated with the existing Career Companion platform</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -234,27 +369,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="56"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -306,27 +421,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -639,19 +745,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultColWidth="17.5546875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42.109375" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="21.88671875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="17.5546875" style="4"/>
+    <col min="1" max="1" width="6.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="42.109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="21.88671875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="17.5546875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
@@ -690,471 +796,774 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="9">
+      <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6">
         <v>46266</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="8" t="s">
+      <c r="F2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="6">
         <v>46266</v>
       </c>
-      <c r="J2" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="8" t="s">
+      <c r="J2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="8">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="9">
+      <c r="B3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6">
         <v>46267</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="8" t="s">
+      <c r="F3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="6">
         <v>46267</v>
       </c>
-      <c r="J3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="8" t="s">
+      <c r="J3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="9">
+      <c r="B4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="6">
         <v>46270</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="8" t="s">
+      <c r="F4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="6">
         <v>46271</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="8" t="s">
+      <c r="J4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="9">
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="6">
         <v>46271</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="8" t="s">
+      <c r="F5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="6">
         <v>46271</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" s="8" t="s">
+      <c r="J5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="9">
+      <c r="B6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="6">
         <v>46273</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="8" t="s">
+      <c r="F6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="6">
         <v>46274</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" s="8" t="s">
+      <c r="J6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+      <c r="A7" s="5">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="9">
+      <c r="B7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="6">
         <v>46275</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="8" t="s">
+      <c r="F7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="6">
         <v>46276</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K7" s="8" t="s">
+      <c r="J7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="10">
+      <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="11">
+      <c r="B8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="8">
         <v>46287</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="10" t="s">
+      <c r="F8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="8">
         <v>46287</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" s="10" t="s">
+      <c r="J8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="A9" s="10">
+      <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="11">
+      <c r="B9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="8">
         <v>46287</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="8">
         <v>46287</v>
       </c>
-      <c r="J9" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K9" s="10" t="s">
+      <c r="J9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="10">
+      <c r="A10" s="7">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="11">
+      <c r="B10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="8">
         <v>46288</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="F10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="8">
         <v>46288</v>
       </c>
-      <c r="J10" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="J10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="10">
+      <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="11">
+      <c r="B11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="8">
         <v>46288</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="F11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="8">
         <v>46288</v>
       </c>
-      <c r="J11" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K11" s="10" t="s">
+      <c r="J11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="6"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="6"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="6"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="6"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="6"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="6"/>
+    <row r="12" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="8">
+        <v>46289</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="8">
+        <v>46289</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A13" s="7">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="8">
+        <v>46289</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="8">
+        <v>46290</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="8">
+        <v>46290</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="8">
+        <v>46290</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46291</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I15" s="8">
+        <v>46291</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="8">
+        <v>46291</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I16" s="8">
+        <v>46292</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="8">
+        <v>46292</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="I17" s="8">
+        <v>46292</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="8">
+        <v>46293</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="I18" s="8">
+        <v>46293</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="8">
+        <v>46293</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" s="8">
+        <v>46294</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="8">
+        <v>46294</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="8">
+        <v>46295</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A21" s="7">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="8">
+        <v>46295</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="I21" s="8">
+        <v>46295</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="A22" s="7">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="8">
+        <v>46296</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="I22" s="8">
+        <v>46296</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="7">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="8">
+        <v>46297</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="I23" s="8">
+        <v>46297</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>104</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1168,7 +1577,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1 G12:G1048576</xm:sqref>
+          <xm:sqref>G1 G24:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1202,7 +1611,7 @@
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1345,18 +1754,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1378,18 +1787,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>